<commit_message>
weekly commit after report generation for the week
</commit_message>
<xml_diff>
--- a/3_output/2026/w23/y2026_w23_weekly_report_output.xlsx
+++ b/3_output/2026/w23/y2026_w23_weekly_report_output.xlsx
@@ -637,7 +637,7 @@
     <t xml:space="preserve">2.4</t>
   </si>
   <si>
-    <t xml:space="preserve">23.2</t>
+    <t xml:space="preserve">5.04</t>
   </si>
   <si>
     <t xml:space="preserve">Week: 23</t>
@@ -2323,10 +2323,10 @@
         <v>18</v>
       </c>
       <c r="C15" s="16" t="n">
-        <v>9.8</v>
+        <v>2.1304</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>13.4</v>
+        <v>2.913</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>0</v>
@@ -2556,32 +2556,32 @@
       <c r="C20" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D20" s="26" t="s">
-        <v>57</v>
+      <c r="D20" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="E20" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="F20" s="26" t="s">
-        <v>57</v>
+      <c r="F20" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="G20" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="H20" s="26" t="s">
-        <v>57</v>
+      <c r="H20" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="I20" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="J20" s="26" t="s">
-        <v>57</v>
+      <c r="J20" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="K20" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="L20" s="26" t="s">
-        <v>57</v>
+      <c r="L20" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="M20" s="14" t="s">
         <v>56</v>
@@ -2619,32 +2619,32 @@
       <c r="C21" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="26" t="s">
-        <v>57</v>
+      <c r="D21" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="E21" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="F21" s="26" t="s">
-        <v>57</v>
+      <c r="F21" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="G21" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="H21" s="26" t="s">
-        <v>57</v>
+      <c r="H21" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="I21" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="J21" s="26" t="s">
-        <v>57</v>
+      <c r="J21" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="K21" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="L21" s="26" t="s">
-        <v>57</v>
+      <c r="L21" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="M21" s="14" t="s">
         <v>57</v>
@@ -2682,32 +2682,32 @@
       <c r="C22" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="D22" s="26" t="s">
-        <v>57</v>
+      <c r="D22" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="E22" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="F22" s="26" t="s">
-        <v>57</v>
+      <c r="F22" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="G22" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="H22" s="26" t="s">
-        <v>57</v>
+      <c r="H22" s="26" t="n">
+        <v>0.02</v>
       </c>
       <c r="I22" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="J22" s="26" t="s">
-        <v>57</v>
+      <c r="J22" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="K22" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="L22" s="26" t="s">
-        <v>57</v>
+      <c r="L22" s="26" t="n">
+        <v>0.01</v>
       </c>
       <c r="M22" s="26" t="s">
         <v>57</v>
@@ -2745,32 +2745,32 @@
       <c r="C23" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="26" t="s">
-        <v>57</v>
+      <c r="D23" s="26" t="n">
+        <v>0.02</v>
       </c>
       <c r="E23" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="26" t="s">
-        <v>57</v>
+      <c r="F23" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="G23" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="H23" s="26" t="s">
-        <v>57</v>
+      <c r="H23" s="26" t="n">
+        <v>0.03</v>
       </c>
       <c r="I23" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="J23" s="26" t="s">
-        <v>57</v>
+      <c r="J23" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="K23" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="L23" s="26" t="s">
-        <v>57</v>
+      <c r="L23" s="26" t="n">
+        <v>0.01</v>
       </c>
       <c r="M23" s="26" t="s">
         <v>57</v>
@@ -2808,32 +2808,32 @@
       <c r="C24" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="26" t="s">
-        <v>57</v>
+      <c r="D24" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="E24" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F24" s="26" t="s">
-        <v>57</v>
+      <c r="F24" s="26" t="n">
+        <v>0.02</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H24" s="26" t="s">
-        <v>57</v>
+      <c r="H24" s="26" t="n">
+        <v>0.08</v>
       </c>
       <c r="I24" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J24" s="26" t="s">
-        <v>57</v>
+      <c r="J24" s="26" t="n">
+        <v>0.02</v>
       </c>
       <c r="K24" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L24" s="26" t="s">
-        <v>57</v>
+      <c r="L24" s="26" t="n">
+        <v>0.04</v>
       </c>
       <c r="M24" s="16" t="s">
         <v>57</v>
@@ -2871,32 +2871,32 @@
       <c r="C25" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="26" t="s">
-        <v>57</v>
+      <c r="D25" s="26" t="n">
+        <v>0.04</v>
       </c>
       <c r="E25" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="26" t="s">
-        <v>57</v>
+      <c r="F25" s="26" t="n">
+        <v>0.08</v>
       </c>
       <c r="G25" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H25" s="26" t="s">
-        <v>57</v>
+      <c r="H25" s="26" t="n">
+        <v>0.34</v>
       </c>
       <c r="I25" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J25" s="26" t="s">
-        <v>57</v>
+      <c r="J25" s="26" t="n">
+        <v>0.11</v>
       </c>
       <c r="K25" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L25" s="26" t="s">
-        <v>57</v>
+      <c r="L25" s="26" t="n">
+        <v>0.17</v>
       </c>
       <c r="M25" s="16" t="s">
         <v>57</v>
@@ -2934,32 +2934,32 @@
       <c r="C26" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D26" s="26" t="s">
-        <v>57</v>
+      <c r="D26" s="26" t="n">
+        <v>0.24</v>
       </c>
       <c r="E26" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="26" t="s">
-        <v>57</v>
+      <c r="F26" s="26" t="n">
+        <v>0.44</v>
       </c>
       <c r="G26" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H26" s="26" t="s">
-        <v>57</v>
+      <c r="H26" s="26" t="n">
+        <v>0.46</v>
       </c>
       <c r="I26" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J26" s="26" t="s">
-        <v>57</v>
+      <c r="J26" s="26" t="n">
+        <v>0.26</v>
       </c>
       <c r="K26" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L26" s="26" t="s">
-        <v>57</v>
+      <c r="L26" s="26" t="n">
+        <v>0.36</v>
       </c>
       <c r="M26" s="16" t="s">
         <v>57</v>
@@ -2997,32 +2997,32 @@
       <c r="C27" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="26" t="s">
-        <v>57</v>
+      <c r="D27" s="26" t="n">
+        <v>0.08</v>
       </c>
       <c r="E27" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F27" s="26" t="s">
-        <v>57</v>
+      <c r="F27" s="26" t="n">
+        <v>0.22</v>
       </c>
       <c r="G27" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H27" s="26" t="s">
-        <v>57</v>
+      <c r="H27" s="26" t="n">
+        <v>0.24</v>
       </c>
       <c r="I27" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J27" s="26" t="s">
-        <v>57</v>
+      <c r="J27" s="26" t="n">
+        <v>0.23</v>
       </c>
       <c r="K27" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L27" s="26" t="s">
-        <v>57</v>
+      <c r="L27" s="26" t="n">
+        <v>0.2</v>
       </c>
       <c r="M27" s="16" t="s">
         <v>57</v>
@@ -3060,32 +3060,32 @@
       <c r="C28" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="26" t="s">
-        <v>57</v>
+      <c r="D28" s="26" t="n">
+        <v>0.18</v>
       </c>
       <c r="E28" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F28" s="26" t="s">
-        <v>57</v>
+      <c r="F28" s="26" t="n">
+        <v>0.16</v>
       </c>
       <c r="G28" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H28" s="26" t="s">
-        <v>57</v>
+      <c r="H28" s="26" t="n">
+        <v>0.57</v>
       </c>
       <c r="I28" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J28" s="26" t="s">
-        <v>57</v>
+      <c r="J28" s="26" t="n">
+        <v>0.16</v>
       </c>
       <c r="K28" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L28" s="26" t="s">
-        <v>57</v>
+      <c r="L28" s="26" t="n">
+        <v>0.31</v>
       </c>
       <c r="M28" s="16" t="s">
         <v>57</v>
@@ -3123,32 +3123,32 @@
       <c r="C29" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="26" t="s">
-        <v>57</v>
+      <c r="D29" s="26" t="n">
+        <v>0.3</v>
       </c>
       <c r="E29" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F29" s="26" t="s">
-        <v>57</v>
+      <c r="F29" s="26" t="n">
+        <v>0.29</v>
       </c>
       <c r="G29" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H29" s="26" t="s">
-        <v>57</v>
+      <c r="H29" s="26" t="n">
+        <v>0.33</v>
       </c>
       <c r="I29" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J29" s="26" t="s">
-        <v>57</v>
+      <c r="J29" s="26" t="n">
+        <v>0.24</v>
       </c>
       <c r="K29" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L29" s="26" t="s">
-        <v>57</v>
+      <c r="L29" s="26" t="n">
+        <v>0.31</v>
       </c>
       <c r="M29" s="16" t="s">
         <v>57</v>
@@ -3186,32 +3186,32 @@
       <c r="C30" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="26" t="s">
-        <v>57</v>
+      <c r="D30" s="26" t="n">
+        <v>0.24</v>
       </c>
       <c r="E30" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F30" s="26" t="s">
-        <v>57</v>
+      <c r="F30" s="26" t="n">
+        <v>0.45</v>
       </c>
       <c r="G30" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H30" s="26" t="s">
-        <v>57</v>
+      <c r="H30" s="26" t="n">
+        <v>0.22</v>
       </c>
       <c r="I30" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J30" s="26" t="s">
-        <v>57</v>
+      <c r="J30" s="26" t="n">
+        <v>0.34</v>
       </c>
       <c r="K30" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L30" s="26" t="s">
-        <v>57</v>
+      <c r="L30" s="26" t="n">
+        <v>0.3</v>
       </c>
       <c r="M30" s="16" t="s">
         <v>57</v>
@@ -3249,32 +3249,32 @@
       <c r="C31" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D31" s="26" t="s">
-        <v>57</v>
+      <c r="D31" s="26" t="n">
+        <v>0.21</v>
       </c>
       <c r="E31" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F31" s="26" t="s">
-        <v>57</v>
+      <c r="F31" s="26" t="n">
+        <v>0.48</v>
       </c>
       <c r="G31" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H31" s="26" t="s">
-        <v>57</v>
+      <c r="H31" s="26" t="n">
+        <v>0.26</v>
       </c>
       <c r="I31" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J31" s="26" t="s">
-        <v>57</v>
+      <c r="J31" s="26" t="n">
+        <v>0.32</v>
       </c>
       <c r="K31" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L31" s="26" t="s">
-        <v>57</v>
+      <c r="L31" s="26" t="n">
+        <v>0.33</v>
       </c>
       <c r="M31" s="16" t="s">
         <v>57</v>
@@ -3312,32 +3312,32 @@
       <c r="C32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D32" s="26" t="s">
-        <v>57</v>
+      <c r="D32" s="26" t="n">
+        <v>0.04</v>
       </c>
       <c r="E32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="26" t="s">
-        <v>57</v>
+      <c r="F32" s="26" t="n">
+        <v>0.19</v>
       </c>
       <c r="G32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H32" s="26" t="s">
-        <v>57</v>
+      <c r="H32" s="26" t="n">
+        <v>0.24</v>
       </c>
       <c r="I32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J32" s="26" t="s">
-        <v>57</v>
+      <c r="J32" s="26" t="n">
+        <v>0.11</v>
       </c>
       <c r="K32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L32" s="26" t="s">
-        <v>57</v>
+      <c r="L32" s="26" t="n">
+        <v>0.16</v>
       </c>
       <c r="M32" s="16" t="s">
         <v>57</v>
@@ -3375,32 +3375,32 @@
       <c r="C33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D33" s="26" t="s">
-        <v>57</v>
+      <c r="D33" s="26" t="n">
+        <v>0.07</v>
       </c>
       <c r="E33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F33" s="26" t="s">
-        <v>57</v>
+      <c r="F33" s="26" t="n">
+        <v>0.08</v>
       </c>
       <c r="G33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H33" s="26" t="s">
-        <v>57</v>
+      <c r="H33" s="26" t="n">
+        <v>0.16</v>
       </c>
       <c r="I33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J33" s="26" t="s">
-        <v>57</v>
+      <c r="J33" s="26" t="n">
+        <v>0.01</v>
       </c>
       <c r="K33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L33" s="26" t="s">
-        <v>57</v>
+      <c r="L33" s="26" t="n">
+        <v>0.11</v>
       </c>
       <c r="M33" s="16" t="s">
         <v>57</v>
@@ -3438,32 +3438,32 @@
       <c r="C34" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D34" s="26" t="s">
-        <v>57</v>
+      <c r="D34" s="26" t="n">
+        <v>0.03</v>
       </c>
       <c r="E34" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F34" s="26" t="s">
-        <v>57</v>
+      <c r="F34" s="26" t="n">
+        <v>0.16</v>
       </c>
       <c r="G34" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H34" s="26" t="s">
-        <v>57</v>
+      <c r="H34" s="26" t="n">
+        <v>0.03</v>
       </c>
       <c r="I34" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J34" s="26" t="s">
-        <v>57</v>
+      <c r="J34" s="26" t="n">
+        <v>0.02</v>
       </c>
       <c r="K34" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L34" s="26" t="s">
-        <v>57</v>
+      <c r="L34" s="26" t="n">
+        <v>0.06</v>
       </c>
       <c r="M34" s="16" t="s">
         <v>57</v>
@@ -4132,16 +4132,16 @@
         <v>116</v>
       </c>
       <c r="F49" s="33" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="G49" s="33" t="n">
-        <v>9.8</v>
+        <v>2.13</v>
       </c>
       <c r="H49" s="33" t="n">
-        <v>13.4</v>
+        <v>2.91</v>
       </c>
       <c r="I49" s="33" t="n">
-        <v>23.2</v>
+        <v>5.04</v>
       </c>
       <c r="J49" s="19"/>
       <c r="K49" s="1"/>
@@ -4360,32 +4360,32 @@
       <c r="C54" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="D54" s="31" t="s">
-        <v>57</v>
+      <c r="D54" s="31" t="n">
+        <v>2.31</v>
       </c>
       <c r="E54" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="F54" s="31" t="s">
-        <v>57</v>
+      <c r="F54" s="31" t="n">
+        <v>3.22</v>
       </c>
       <c r="G54" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="H54" s="31" t="s">
-        <v>57</v>
+      <c r="H54" s="31" t="n">
+        <v>2.85</v>
       </c>
       <c r="I54" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="J54" s="31" t="s">
-        <v>57</v>
+      <c r="J54" s="31" t="n">
+        <v>2.58</v>
       </c>
       <c r="K54" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="L54" s="31" t="s">
-        <v>57</v>
+      <c r="L54" s="31" t="n">
+        <v>2.77</v>
       </c>
       <c r="M54" s="31" t="s">
         <v>63</v>
@@ -4423,32 +4423,32 @@
       <c r="C55" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="D55" s="31" t="s">
-        <v>57</v>
+      <c r="D55" s="31" t="n">
+        <v>3.22</v>
       </c>
       <c r="E55" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="F55" s="31" t="s">
-        <v>57</v>
+      <c r="F55" s="31" t="n">
+        <v>4.14</v>
       </c>
       <c r="G55" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="H55" s="31" t="s">
-        <v>57</v>
+      <c r="H55" s="31" t="n">
+        <v>5.07</v>
       </c>
       <c r="I55" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="J55" s="31" t="s">
-        <v>57</v>
+      <c r="J55" s="31" t="n">
+        <v>2.89</v>
       </c>
       <c r="K55" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="L55" s="31" t="s">
-        <v>57</v>
+      <c r="L55" s="31" t="n">
+        <v>4.01</v>
       </c>
       <c r="M55" s="32" t="s">
         <v>57</v>
@@ -4486,32 +4486,32 @@
       <c r="C56" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="D56" s="31" t="s">
-        <v>57</v>
+      <c r="D56" s="31" t="n">
+        <v>7.42</v>
       </c>
       <c r="E56" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="F56" s="31" t="s">
-        <v>57</v>
+      <c r="F56" s="31" t="n">
+        <v>16.14</v>
       </c>
       <c r="G56" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="H56" s="31" t="s">
-        <v>57</v>
+      <c r="H56" s="31" t="n">
+        <v>22.29</v>
       </c>
       <c r="I56" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="J56" s="31" t="s">
-        <v>57</v>
+      <c r="J56" s="31" t="n">
+        <v>5.55</v>
       </c>
       <c r="K56" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="L56" s="31" t="s">
-        <v>57</v>
+      <c r="L56" s="31" t="n">
+        <v>14.24</v>
       </c>
       <c r="M56" s="32" t="s">
         <v>57</v>
@@ -4549,32 +4549,32 @@
       <c r="C57" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="D57" s="31" t="s">
-        <v>57</v>
+      <c r="D57" s="31" t="n">
+        <v>35.89</v>
       </c>
       <c r="E57" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="F57" s="31" t="s">
-        <v>57</v>
+      <c r="F57" s="31" t="n">
+        <v>48.9</v>
       </c>
       <c r="G57" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="H57" s="31" t="s">
-        <v>57</v>
+      <c r="H57" s="31" t="n">
+        <v>62.77</v>
       </c>
       <c r="I57" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="J57" s="31" t="s">
-        <v>57</v>
+      <c r="J57" s="31" t="n">
+        <v>26.09</v>
       </c>
       <c r="K57" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="L57" s="31" t="s">
-        <v>57</v>
+      <c r="L57" s="31" t="n">
+        <v>46.27</v>
       </c>
       <c r="M57" s="32" t="s">
         <v>57</v>
@@ -4612,32 +4612,32 @@
       <c r="C58" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D58" s="31" t="s">
-        <v>57</v>
+      <c r="D58" s="31" t="n">
+        <v>29.29</v>
       </c>
       <c r="E58" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F58" s="31" t="s">
-        <v>57</v>
+      <c r="F58" s="31" t="n">
+        <v>89.14</v>
       </c>
       <c r="G58" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H58" s="31" t="s">
-        <v>57</v>
+      <c r="H58" s="31" t="n">
+        <v>117.32</v>
       </c>
       <c r="I58" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J58" s="31" t="s">
-        <v>57</v>
+      <c r="J58" s="31" t="n">
+        <v>25.91</v>
       </c>
       <c r="K58" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L58" s="31" t="s">
-        <v>57</v>
+      <c r="L58" s="31" t="n">
+        <v>73.21</v>
       </c>
       <c r="M58" s="33" t="s">
         <v>57</v>
@@ -4675,32 +4675,32 @@
       <c r="C59" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D59" s="31" t="s">
-        <v>57</v>
+      <c r="D59" s="31" t="n">
+        <v>64.7</v>
       </c>
       <c r="E59" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F59" s="31" t="s">
-        <v>57</v>
+      <c r="F59" s="31" t="n">
+        <v>101.22</v>
       </c>
       <c r="G59" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H59" s="31" t="s">
-        <v>57</v>
+      <c r="H59" s="31" t="n">
+        <v>170.25</v>
       </c>
       <c r="I59" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J59" s="31" t="s">
-        <v>57</v>
+      <c r="J59" s="31" t="n">
+        <v>85.92</v>
       </c>
       <c r="K59" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L59" s="31" t="s">
-        <v>57</v>
+      <c r="L59" s="31" t="n">
+        <v>115.14</v>
       </c>
       <c r="M59" s="33" t="s">
         <v>57</v>
@@ -4738,32 +4738,32 @@
       <c r="C60" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D60" s="31" t="s">
-        <v>57</v>
+      <c r="D60" s="31" t="n">
+        <v>92.44</v>
       </c>
       <c r="E60" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F60" s="31" t="s">
-        <v>57</v>
+      <c r="F60" s="31" t="n">
+        <v>182.39</v>
       </c>
       <c r="G60" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H60" s="31" t="s">
-        <v>57</v>
+      <c r="H60" s="31" t="n">
+        <v>160.99</v>
       </c>
       <c r="I60" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J60" s="31" t="s">
-        <v>57</v>
+      <c r="J60" s="31" t="n">
+        <v>79.76</v>
       </c>
       <c r="K60" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L60" s="31" t="s">
-        <v>57</v>
+      <c r="L60" s="31" t="n">
+        <v>135.15</v>
       </c>
       <c r="M60" s="33" t="s">
         <v>57</v>
@@ -4801,32 +4801,32 @@
       <c r="C61" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D61" s="31" t="s">
-        <v>57</v>
+      <c r="D61" s="31" t="n">
+        <v>46.26</v>
       </c>
       <c r="E61" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F61" s="31" t="s">
-        <v>57</v>
+      <c r="F61" s="31" t="n">
+        <v>133.22</v>
       </c>
       <c r="G61" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H61" s="31" t="s">
-        <v>57</v>
+      <c r="H61" s="31" t="n">
+        <v>81.37</v>
       </c>
       <c r="I61" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J61" s="31" t="s">
-        <v>57</v>
+      <c r="J61" s="31" t="n">
+        <v>50.29</v>
       </c>
       <c r="K61" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L61" s="31" t="s">
-        <v>57</v>
+      <c r="L61" s="31" t="n">
+        <v>79.9</v>
       </c>
       <c r="M61" s="33" t="s">
         <v>57</v>
@@ -4864,32 +4864,32 @@
       <c r="C62" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D62" s="31" t="s">
-        <v>57</v>
+      <c r="D62" s="31" t="n">
+        <v>28.44</v>
       </c>
       <c r="E62" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F62" s="31" t="s">
-        <v>57</v>
+      <c r="F62" s="31" t="n">
+        <v>77.88</v>
       </c>
       <c r="G62" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H62" s="31" t="s">
-        <v>57</v>
+      <c r="H62" s="31" t="n">
+        <v>74.94</v>
       </c>
       <c r="I62" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J62" s="31" t="s">
-        <v>57</v>
+      <c r="J62" s="31" t="n">
+        <v>22.2</v>
       </c>
       <c r="K62" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L62" s="31" t="s">
-        <v>57</v>
+      <c r="L62" s="31" t="n">
+        <v>54.45</v>
       </c>
       <c r="M62" s="33" t="s">
         <v>57</v>
@@ -4927,32 +4927,32 @@
       <c r="C63" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D63" s="31" t="s">
-        <v>57</v>
+      <c r="D63" s="31" t="n">
+        <v>28.98</v>
       </c>
       <c r="E63" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F63" s="31" t="s">
-        <v>57</v>
+      <c r="F63" s="31" t="n">
+        <v>84.16</v>
       </c>
       <c r="G63" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H63" s="31" t="s">
-        <v>57</v>
+      <c r="H63" s="31" t="n">
+        <v>41.36</v>
       </c>
       <c r="I63" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J63" s="31" t="s">
-        <v>57</v>
+      <c r="J63" s="31" t="n">
+        <v>33.16</v>
       </c>
       <c r="K63" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L63" s="31" t="s">
-        <v>57</v>
+      <c r="L63" s="31" t="n">
+        <v>47.21</v>
       </c>
       <c r="M63" s="33" t="s">
         <v>57</v>
@@ -4990,32 +4990,32 @@
       <c r="C64" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D64" s="31" t="s">
-        <v>57</v>
+      <c r="D64" s="31" t="n">
+        <v>20.07</v>
       </c>
       <c r="E64" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F64" s="31" t="s">
-        <v>57</v>
+      <c r="F64" s="31" t="n">
+        <v>60.06</v>
       </c>
       <c r="G64" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H64" s="31" t="s">
-        <v>57</v>
+      <c r="H64" s="31" t="n">
+        <v>32.32</v>
       </c>
       <c r="I64" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J64" s="31" t="s">
-        <v>57</v>
+      <c r="J64" s="31" t="n">
+        <v>25.24</v>
       </c>
       <c r="K64" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L64" s="31" t="s">
-        <v>57</v>
+      <c r="L64" s="31" t="n">
+        <v>34.73</v>
       </c>
       <c r="M64" s="33" t="s">
         <v>57</v>
@@ -5053,32 +5053,32 @@
       <c r="C65" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D65" s="31" t="s">
-        <v>57</v>
+      <c r="D65" s="31" t="n">
+        <v>22.49</v>
       </c>
       <c r="E65" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F65" s="31" t="s">
-        <v>57</v>
+      <c r="F65" s="31" t="n">
+        <v>72.68</v>
       </c>
       <c r="G65" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H65" s="31" t="s">
-        <v>57</v>
+      <c r="H65" s="31" t="n">
+        <v>32.85</v>
       </c>
       <c r="I65" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J65" s="31" t="s">
-        <v>57</v>
+      <c r="J65" s="31" t="n">
+        <v>20.8</v>
       </c>
       <c r="K65" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L65" s="31" t="s">
-        <v>57</v>
+      <c r="L65" s="31" t="n">
+        <v>37.56</v>
       </c>
       <c r="M65" s="33" t="s">
         <v>57</v>
@@ -5116,32 +5116,32 @@
       <c r="C66" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D66" s="31" t="s">
-        <v>57</v>
+      <c r="D66" s="31" t="n">
+        <v>9.31</v>
       </c>
       <c r="E66" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F66" s="31" t="s">
-        <v>57</v>
+      <c r="F66" s="31" t="n">
+        <v>26.92</v>
       </c>
       <c r="G66" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H66" s="31" t="s">
-        <v>57</v>
+      <c r="H66" s="31" t="n">
+        <v>22.11</v>
       </c>
       <c r="I66" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J66" s="31" t="s">
-        <v>57</v>
+      <c r="J66" s="31" t="n">
+        <v>9.27</v>
       </c>
       <c r="K66" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L66" s="31" t="s">
-        <v>57</v>
+      <c r="L66" s="31" t="n">
+        <v>17.86</v>
       </c>
       <c r="M66" s="33" t="s">
         <v>57</v>
@@ -5179,32 +5179,32 @@
       <c r="C67" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D67" s="31" t="s">
-        <v>57</v>
+      <c r="D67" s="31" t="n">
+        <v>4.5</v>
       </c>
       <c r="E67" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F67" s="31" t="s">
-        <v>57</v>
+      <c r="F67" s="31" t="n">
+        <v>40.22</v>
       </c>
       <c r="G67" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H67" s="31" t="s">
-        <v>57</v>
+      <c r="H67" s="31" t="n">
+        <v>16.83</v>
       </c>
       <c r="I67" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J67" s="31" t="s">
-        <v>57</v>
+      <c r="J67" s="31" t="n">
+        <v>5.09</v>
       </c>
       <c r="K67" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L67" s="31" t="s">
-        <v>57</v>
+      <c r="L67" s="31" t="n">
+        <v>17.26</v>
       </c>
       <c r="M67" s="33" t="s">
         <v>57</v>
@@ -5242,32 +5242,32 @@
       <c r="C68" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D68" s="31" t="s">
-        <v>57</v>
+      <c r="D68" s="31" t="n">
+        <v>2.76</v>
       </c>
       <c r="E68" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="F68" s="31" t="s">
-        <v>57</v>
+      <c r="F68" s="31" t="n">
+        <v>38.26</v>
       </c>
       <c r="G68" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="H68" s="31" t="s">
-        <v>57</v>
+      <c r="H68" s="31" t="n">
+        <v>9.25</v>
       </c>
       <c r="I68" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="J68" s="31" t="s">
-        <v>57</v>
+      <c r="J68" s="31" t="n">
+        <v>2.92</v>
       </c>
       <c r="K68" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="L68" s="31" t="s">
-        <v>57</v>
+      <c r="L68" s="31" t="n">
+        <v>13.36</v>
       </c>
       <c r="M68" s="33" t="s">
         <v>57</v>
@@ -41371,10 +41371,10 @@
         <v>86</v>
       </c>
       <c r="B10" t="n">
-        <v>9.8</v>
+        <v>2.1304</v>
       </c>
       <c r="C10" t="n">
-        <v>13.4</v>
+        <v>2.913</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -41454,32 +41454,32 @@
       <c r="B2" t="s">
         <v>56</v>
       </c>
-      <c r="C2" t="s">
-        <v>57</v>
+      <c r="C2" t="n">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>56</v>
       </c>
-      <c r="E2" t="s">
-        <v>57</v>
+      <c r="E2" t="n">
+        <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>56</v>
       </c>
-      <c r="G2" t="s">
-        <v>57</v>
+      <c r="G2" t="n">
+        <v>0</v>
       </c>
       <c r="H2" t="s">
         <v>56</v>
       </c>
-      <c r="I2" t="s">
-        <v>57</v>
+      <c r="I2" t="n">
+        <v>0</v>
       </c>
       <c r="J2" t="s">
         <v>56</v>
       </c>
-      <c r="K2" t="s">
-        <v>57</v>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
       <c r="L2" t="s">
         <v>56</v>
@@ -41498,32 +41498,32 @@
       <c r="B3" t="s">
         <v>57</v>
       </c>
-      <c r="C3" t="s">
-        <v>57</v>
+      <c r="C3" t="n">
+        <v>0</v>
       </c>
       <c r="D3" t="s">
         <v>57</v>
       </c>
-      <c r="E3" t="s">
-        <v>57</v>
+      <c r="E3" t="n">
+        <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>57</v>
       </c>
-      <c r="G3" t="s">
-        <v>57</v>
+      <c r="G3" t="n">
+        <v>0</v>
       </c>
       <c r="H3" t="s">
         <v>57</v>
       </c>
-      <c r="I3" t="s">
-        <v>57</v>
+      <c r="I3" t="n">
+        <v>0</v>
       </c>
       <c r="J3" t="s">
         <v>57</v>
       </c>
-      <c r="K3" t="s">
-        <v>57</v>
+      <c r="K3" t="n">
+        <v>0</v>
       </c>
       <c r="L3" t="s">
         <v>57</v>
@@ -41542,32 +41542,32 @@
       <c r="B4" t="s">
         <v>57</v>
       </c>
-      <c r="C4" t="s">
-        <v>57</v>
+      <c r="C4" t="n">
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>57</v>
       </c>
-      <c r="E4" t="s">
-        <v>57</v>
+      <c r="E4" t="n">
+        <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>57</v>
       </c>
-      <c r="G4" t="s">
-        <v>57</v>
+      <c r="G4" t="n">
+        <v>0.02</v>
       </c>
       <c r="H4" t="s">
         <v>57</v>
       </c>
-      <c r="I4" t="s">
-        <v>57</v>
+      <c r="I4" t="n">
+        <v>0</v>
       </c>
       <c r="J4" t="s">
         <v>57</v>
       </c>
-      <c r="K4" t="s">
-        <v>57</v>
+      <c r="K4" t="n">
+        <v>0.01</v>
       </c>
       <c r="L4" t="s">
         <v>57</v>
@@ -41586,32 +41586,32 @@
       <c r="B5" t="s">
         <v>57</v>
       </c>
-      <c r="C5" t="s">
-        <v>57</v>
+      <c r="C5" t="n">
+        <v>0.02</v>
       </c>
       <c r="D5" t="s">
         <v>57</v>
       </c>
-      <c r="E5" t="s">
-        <v>57</v>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>57</v>
       </c>
-      <c r="G5" t="s">
-        <v>57</v>
+      <c r="G5" t="n">
+        <v>0.03</v>
       </c>
       <c r="H5" t="s">
         <v>57</v>
       </c>
-      <c r="I5" t="s">
-        <v>57</v>
+      <c r="I5" t="n">
+        <v>0</v>
       </c>
       <c r="J5" t="s">
         <v>57</v>
       </c>
-      <c r="K5" t="s">
-        <v>57</v>
+      <c r="K5" t="n">
+        <v>0.01</v>
       </c>
       <c r="L5" t="s">
         <v>57</v>
@@ -41630,32 +41630,32 @@
       <c r="B6" t="s">
         <v>57</v>
       </c>
-      <c r="C6" t="s">
-        <v>57</v>
+      <c r="C6" t="n">
+        <v>0</v>
       </c>
       <c r="D6" t="s">
         <v>57</v>
       </c>
-      <c r="E6" t="s">
-        <v>57</v>
+      <c r="E6" t="n">
+        <v>0.02</v>
       </c>
       <c r="F6" t="s">
         <v>57</v>
       </c>
-      <c r="G6" t="s">
-        <v>57</v>
+      <c r="G6" t="n">
+        <v>0.08</v>
       </c>
       <c r="H6" t="s">
         <v>57</v>
       </c>
-      <c r="I6" t="s">
-        <v>57</v>
+      <c r="I6" t="n">
+        <v>0.02</v>
       </c>
       <c r="J6" t="s">
         <v>57</v>
       </c>
-      <c r="K6" t="s">
-        <v>57</v>
+      <c r="K6" t="n">
+        <v>0.04</v>
       </c>
       <c r="L6" t="s">
         <v>57</v>
@@ -41674,32 +41674,32 @@
       <c r="B7" t="s">
         <v>57</v>
       </c>
-      <c r="C7" t="s">
-        <v>57</v>
+      <c r="C7" t="n">
+        <v>0.04</v>
       </c>
       <c r="D7" t="s">
         <v>57</v>
       </c>
-      <c r="E7" t="s">
-        <v>57</v>
+      <c r="E7" t="n">
+        <v>0.08</v>
       </c>
       <c r="F7" t="s">
         <v>57</v>
       </c>
-      <c r="G7" t="s">
-        <v>57</v>
+      <c r="G7" t="n">
+        <v>0.34</v>
       </c>
       <c r="H7" t="s">
         <v>57</v>
       </c>
-      <c r="I7" t="s">
-        <v>57</v>
+      <c r="I7" t="n">
+        <v>0.11</v>
       </c>
       <c r="J7" t="s">
         <v>57</v>
       </c>
-      <c r="K7" t="s">
-        <v>57</v>
+      <c r="K7" t="n">
+        <v>0.17</v>
       </c>
       <c r="L7" t="s">
         <v>57</v>
@@ -41718,32 +41718,32 @@
       <c r="B8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" t="s">
-        <v>57</v>
+      <c r="C8" t="n">
+        <v>0.24</v>
       </c>
       <c r="D8" t="s">
         <v>57</v>
       </c>
-      <c r="E8" t="s">
-        <v>57</v>
+      <c r="E8" t="n">
+        <v>0.44</v>
       </c>
       <c r="F8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
-        <v>57</v>
+      <c r="G8" t="n">
+        <v>0.46</v>
       </c>
       <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="I8" t="s">
-        <v>57</v>
+      <c r="I8" t="n">
+        <v>0.26</v>
       </c>
       <c r="J8" t="s">
         <v>57</v>
       </c>
-      <c r="K8" t="s">
-        <v>57</v>
+      <c r="K8" t="n">
+        <v>0.36</v>
       </c>
       <c r="L8" t="s">
         <v>57</v>
@@ -41762,32 +41762,32 @@
       <c r="B9" t="s">
         <v>57</v>
       </c>
-      <c r="C9" t="s">
-        <v>57</v>
+      <c r="C9" t="n">
+        <v>0.08</v>
       </c>
       <c r="D9" t="s">
         <v>57</v>
       </c>
-      <c r="E9" t="s">
-        <v>57</v>
+      <c r="E9" t="n">
+        <v>0.22</v>
       </c>
       <c r="F9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
-        <v>57</v>
+      <c r="G9" t="n">
+        <v>0.24</v>
       </c>
       <c r="H9" t="s">
         <v>57</v>
       </c>
-      <c r="I9" t="s">
-        <v>57</v>
+      <c r="I9" t="n">
+        <v>0.23</v>
       </c>
       <c r="J9" t="s">
         <v>57</v>
       </c>
-      <c r="K9" t="s">
-        <v>57</v>
+      <c r="K9" t="n">
+        <v>0.2</v>
       </c>
       <c r="L9" t="s">
         <v>57</v>
@@ -41806,32 +41806,32 @@
       <c r="B10" t="s">
         <v>57</v>
       </c>
-      <c r="C10" t="s">
-        <v>57</v>
+      <c r="C10" t="n">
+        <v>0.18</v>
       </c>
       <c r="D10" t="s">
         <v>57</v>
       </c>
-      <c r="E10" t="s">
-        <v>57</v>
+      <c r="E10" t="n">
+        <v>0.16</v>
       </c>
       <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="G10" t="s">
-        <v>57</v>
+      <c r="G10" t="n">
+        <v>0.57</v>
       </c>
       <c r="H10" t="s">
         <v>57</v>
       </c>
-      <c r="I10" t="s">
-        <v>57</v>
+      <c r="I10" t="n">
+        <v>0.16</v>
       </c>
       <c r="J10" t="s">
         <v>57</v>
       </c>
-      <c r="K10" t="s">
-        <v>57</v>
+      <c r="K10" t="n">
+        <v>0.31</v>
       </c>
       <c r="L10" t="s">
         <v>57</v>
@@ -41850,32 +41850,32 @@
       <c r="B11" t="s">
         <v>57</v>
       </c>
-      <c r="C11" t="s">
-        <v>57</v>
+      <c r="C11" t="n">
+        <v>0.3</v>
       </c>
       <c r="D11" t="s">
         <v>57</v>
       </c>
-      <c r="E11" t="s">
-        <v>57</v>
+      <c r="E11" t="n">
+        <v>0.29</v>
       </c>
       <c r="F11" t="s">
         <v>57</v>
       </c>
-      <c r="G11" t="s">
-        <v>57</v>
+      <c r="G11" t="n">
+        <v>0.33</v>
       </c>
       <c r="H11" t="s">
         <v>57</v>
       </c>
-      <c r="I11" t="s">
-        <v>57</v>
+      <c r="I11" t="n">
+        <v>0.24</v>
       </c>
       <c r="J11" t="s">
         <v>57</v>
       </c>
-      <c r="K11" t="s">
-        <v>57</v>
+      <c r="K11" t="n">
+        <v>0.31</v>
       </c>
       <c r="L11" t="s">
         <v>57</v>
@@ -41894,32 +41894,32 @@
       <c r="B12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
-        <v>57</v>
+      <c r="C12" t="n">
+        <v>0.24</v>
       </c>
       <c r="D12" t="s">
         <v>57</v>
       </c>
-      <c r="E12" t="s">
-        <v>57</v>
+      <c r="E12" t="n">
+        <v>0.45</v>
       </c>
       <c r="F12" t="s">
         <v>57</v>
       </c>
-      <c r="G12" t="s">
-        <v>57</v>
+      <c r="G12" t="n">
+        <v>0.22</v>
       </c>
       <c r="H12" t="s">
         <v>57</v>
       </c>
-      <c r="I12" t="s">
-        <v>57</v>
+      <c r="I12" t="n">
+        <v>0.34</v>
       </c>
       <c r="J12" t="s">
         <v>57</v>
       </c>
-      <c r="K12" t="s">
-        <v>57</v>
+      <c r="K12" t="n">
+        <v>0.3</v>
       </c>
       <c r="L12" t="s">
         <v>57</v>
@@ -41938,32 +41938,32 @@
       <c r="B13" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
-        <v>57</v>
+      <c r="C13" t="n">
+        <v>0.21</v>
       </c>
       <c r="D13" t="s">
         <v>57</v>
       </c>
-      <c r="E13" t="s">
-        <v>57</v>
+      <c r="E13" t="n">
+        <v>0.48</v>
       </c>
       <c r="F13" t="s">
         <v>57</v>
       </c>
-      <c r="G13" t="s">
-        <v>57</v>
+      <c r="G13" t="n">
+        <v>0.26</v>
       </c>
       <c r="H13" t="s">
         <v>57</v>
       </c>
-      <c r="I13" t="s">
-        <v>57</v>
+      <c r="I13" t="n">
+        <v>0.32</v>
       </c>
       <c r="J13" t="s">
         <v>57</v>
       </c>
-      <c r="K13" t="s">
-        <v>57</v>
+      <c r="K13" t="n">
+        <v>0.33</v>
       </c>
       <c r="L13" t="s">
         <v>57</v>
@@ -41982,32 +41982,32 @@
       <c r="B14" t="s">
         <v>57</v>
       </c>
-      <c r="C14" t="s">
-        <v>57</v>
+      <c r="C14" t="n">
+        <v>0.04</v>
       </c>
       <c r="D14" t="s">
         <v>57</v>
       </c>
-      <c r="E14" t="s">
-        <v>57</v>
+      <c r="E14" t="n">
+        <v>0.19</v>
       </c>
       <c r="F14" t="s">
         <v>57</v>
       </c>
-      <c r="G14" t="s">
-        <v>57</v>
+      <c r="G14" t="n">
+        <v>0.24</v>
       </c>
       <c r="H14" t="s">
         <v>57</v>
       </c>
-      <c r="I14" t="s">
-        <v>57</v>
+      <c r="I14" t="n">
+        <v>0.11</v>
       </c>
       <c r="J14" t="s">
         <v>57</v>
       </c>
-      <c r="K14" t="s">
-        <v>57</v>
+      <c r="K14" t="n">
+        <v>0.16</v>
       </c>
       <c r="L14" t="s">
         <v>57</v>
@@ -42026,32 +42026,32 @@
       <c r="B15" t="s">
         <v>57</v>
       </c>
-      <c r="C15" t="s">
-        <v>57</v>
+      <c r="C15" t="n">
+        <v>0.07</v>
       </c>
       <c r="D15" t="s">
         <v>57</v>
       </c>
-      <c r="E15" t="s">
-        <v>57</v>
+      <c r="E15" t="n">
+        <v>0.08</v>
       </c>
       <c r="F15" t="s">
         <v>57</v>
       </c>
-      <c r="G15" t="s">
-        <v>57</v>
+      <c r="G15" t="n">
+        <v>0.16</v>
       </c>
       <c r="H15" t="s">
         <v>57</v>
       </c>
-      <c r="I15" t="s">
-        <v>57</v>
+      <c r="I15" t="n">
+        <v>0.01</v>
       </c>
       <c r="J15" t="s">
         <v>57</v>
       </c>
-      <c r="K15" t="s">
-        <v>57</v>
+      <c r="K15" t="n">
+        <v>0.11</v>
       </c>
       <c r="L15" t="s">
         <v>57</v>
@@ -42070,32 +42070,32 @@
       <c r="B16" t="s">
         <v>57</v>
       </c>
-      <c r="C16" t="s">
-        <v>57</v>
+      <c r="C16" t="n">
+        <v>0.03</v>
       </c>
       <c r="D16" t="s">
         <v>57</v>
       </c>
-      <c r="E16" t="s">
-        <v>57</v>
+      <c r="E16" t="n">
+        <v>0.16</v>
       </c>
       <c r="F16" t="s">
         <v>57</v>
       </c>
-      <c r="G16" t="s">
-        <v>57</v>
+      <c r="G16" t="n">
+        <v>0.03</v>
       </c>
       <c r="H16" t="s">
         <v>57</v>
       </c>
-      <c r="I16" t="s">
-        <v>57</v>
+      <c r="I16" t="n">
+        <v>0.02</v>
       </c>
       <c r="J16" t="s">
         <v>57</v>
       </c>
-      <c r="K16" t="s">
-        <v>57</v>
+      <c r="K16" t="n">
+        <v>0.06</v>
       </c>
       <c r="L16" t="s">
         <v>57</v>
@@ -42350,16 +42350,16 @@
         <v>116</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>9.8</v>
+        <v>2.13</v>
       </c>
       <c r="G10" t="n">
-        <v>13.4</v>
+        <v>2.91</v>
       </c>
       <c r="H10" t="n">
-        <v>23.2</v>
+        <v>5.04</v>
       </c>
     </row>
   </sheetData>
@@ -42424,32 +42424,32 @@
       <c r="B2" t="s">
         <v>58</v>
       </c>
-      <c r="C2" t="s">
-        <v>57</v>
+      <c r="C2" t="n">
+        <v>2.31</v>
       </c>
       <c r="D2" t="s">
         <v>59</v>
       </c>
-      <c r="E2" t="s">
-        <v>57</v>
+      <c r="E2" t="n">
+        <v>3.22</v>
       </c>
       <c r="F2" t="s">
         <v>60</v>
       </c>
-      <c r="G2" t="s">
-        <v>57</v>
+      <c r="G2" t="n">
+        <v>2.85</v>
       </c>
       <c r="H2" t="s">
         <v>61</v>
       </c>
-      <c r="I2" t="s">
-        <v>57</v>
+      <c r="I2" t="n">
+        <v>2.58</v>
       </c>
       <c r="J2" t="s">
         <v>62</v>
       </c>
-      <c r="K2" t="s">
-        <v>57</v>
+      <c r="K2" t="n">
+        <v>2.77</v>
       </c>
       <c r="L2" t="s">
         <v>63</v>
@@ -42468,32 +42468,32 @@
       <c r="B3" t="s">
         <v>57</v>
       </c>
-      <c r="C3" t="s">
-        <v>57</v>
+      <c r="C3" t="n">
+        <v>3.22</v>
       </c>
       <c r="D3" t="s">
         <v>57</v>
       </c>
-      <c r="E3" t="s">
-        <v>57</v>
+      <c r="E3" t="n">
+        <v>4.14</v>
       </c>
       <c r="F3" t="s">
         <v>57</v>
       </c>
-      <c r="G3" t="s">
-        <v>57</v>
+      <c r="G3" t="n">
+        <v>5.07</v>
       </c>
       <c r="H3" t="s">
         <v>57</v>
       </c>
-      <c r="I3" t="s">
-        <v>57</v>
+      <c r="I3" t="n">
+        <v>2.89</v>
       </c>
       <c r="J3" t="s">
         <v>57</v>
       </c>
-      <c r="K3" t="s">
-        <v>57</v>
+      <c r="K3" t="n">
+        <v>4.01</v>
       </c>
       <c r="L3" t="s">
         <v>57</v>
@@ -42512,32 +42512,32 @@
       <c r="B4" t="s">
         <v>57</v>
       </c>
-      <c r="C4" t="s">
-        <v>57</v>
+      <c r="C4" t="n">
+        <v>7.42</v>
       </c>
       <c r="D4" t="s">
         <v>57</v>
       </c>
-      <c r="E4" t="s">
-        <v>57</v>
+      <c r="E4" t="n">
+        <v>16.14</v>
       </c>
       <c r="F4" t="s">
         <v>57</v>
       </c>
-      <c r="G4" t="s">
-        <v>57</v>
+      <c r="G4" t="n">
+        <v>22.29</v>
       </c>
       <c r="H4" t="s">
         <v>57</v>
       </c>
-      <c r="I4" t="s">
-        <v>57</v>
+      <c r="I4" t="n">
+        <v>5.55</v>
       </c>
       <c r="J4" t="s">
         <v>57</v>
       </c>
-      <c r="K4" t="s">
-        <v>57</v>
+      <c r="K4" t="n">
+        <v>14.24</v>
       </c>
       <c r="L4" t="s">
         <v>57</v>
@@ -42556,32 +42556,32 @@
       <c r="B5" t="s">
         <v>57</v>
       </c>
-      <c r="C5" t="s">
-        <v>57</v>
+      <c r="C5" t="n">
+        <v>35.89</v>
       </c>
       <c r="D5" t="s">
         <v>57</v>
       </c>
-      <c r="E5" t="s">
-        <v>57</v>
+      <c r="E5" t="n">
+        <v>48.9</v>
       </c>
       <c r="F5" t="s">
         <v>57</v>
       </c>
-      <c r="G5" t="s">
-        <v>57</v>
+      <c r="G5" t="n">
+        <v>62.77</v>
       </c>
       <c r="H5" t="s">
         <v>57</v>
       </c>
-      <c r="I5" t="s">
-        <v>57</v>
+      <c r="I5" t="n">
+        <v>26.09</v>
       </c>
       <c r="J5" t="s">
         <v>57</v>
       </c>
-      <c r="K5" t="s">
-        <v>57</v>
+      <c r="K5" t="n">
+        <v>46.27</v>
       </c>
       <c r="L5" t="s">
         <v>57</v>
@@ -42600,32 +42600,32 @@
       <c r="B6" t="s">
         <v>57</v>
       </c>
-      <c r="C6" t="s">
-        <v>57</v>
+      <c r="C6" t="n">
+        <v>29.29</v>
       </c>
       <c r="D6" t="s">
         <v>57</v>
       </c>
-      <c r="E6" t="s">
-        <v>57</v>
+      <c r="E6" t="n">
+        <v>89.14</v>
       </c>
       <c r="F6" t="s">
         <v>57</v>
       </c>
-      <c r="G6" t="s">
-        <v>57</v>
+      <c r="G6" t="n">
+        <v>117.32</v>
       </c>
       <c r="H6" t="s">
         <v>57</v>
       </c>
-      <c r="I6" t="s">
-        <v>57</v>
+      <c r="I6" t="n">
+        <v>25.91</v>
       </c>
       <c r="J6" t="s">
         <v>57</v>
       </c>
-      <c r="K6" t="s">
-        <v>57</v>
+      <c r="K6" t="n">
+        <v>73.21</v>
       </c>
       <c r="L6" t="s">
         <v>57</v>
@@ -42644,32 +42644,32 @@
       <c r="B7" t="s">
         <v>57</v>
       </c>
-      <c r="C7" t="s">
-        <v>57</v>
+      <c r="C7" t="n">
+        <v>64.7</v>
       </c>
       <c r="D7" t="s">
         <v>57</v>
       </c>
-      <c r="E7" t="s">
-        <v>57</v>
+      <c r="E7" t="n">
+        <v>101.22</v>
       </c>
       <c r="F7" t="s">
         <v>57</v>
       </c>
-      <c r="G7" t="s">
-        <v>57</v>
+      <c r="G7" t="n">
+        <v>170.25</v>
       </c>
       <c r="H7" t="s">
         <v>57</v>
       </c>
-      <c r="I7" t="s">
-        <v>57</v>
+      <c r="I7" t="n">
+        <v>85.92</v>
       </c>
       <c r="J7" t="s">
         <v>57</v>
       </c>
-      <c r="K7" t="s">
-        <v>57</v>
+      <c r="K7" t="n">
+        <v>115.14</v>
       </c>
       <c r="L7" t="s">
         <v>57</v>
@@ -42688,32 +42688,32 @@
       <c r="B8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" t="s">
-        <v>57</v>
+      <c r="C8" t="n">
+        <v>92.44</v>
       </c>
       <c r="D8" t="s">
         <v>57</v>
       </c>
-      <c r="E8" t="s">
-        <v>57</v>
+      <c r="E8" t="n">
+        <v>182.39</v>
       </c>
       <c r="F8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
-        <v>57</v>
+      <c r="G8" t="n">
+        <v>160.99</v>
       </c>
       <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="I8" t="s">
-        <v>57</v>
+      <c r="I8" t="n">
+        <v>79.76</v>
       </c>
       <c r="J8" t="s">
         <v>57</v>
       </c>
-      <c r="K8" t="s">
-        <v>57</v>
+      <c r="K8" t="n">
+        <v>135.15</v>
       </c>
       <c r="L8" t="s">
         <v>57</v>
@@ -42732,32 +42732,32 @@
       <c r="B9" t="s">
         <v>57</v>
       </c>
-      <c r="C9" t="s">
-        <v>57</v>
+      <c r="C9" t="n">
+        <v>46.26</v>
       </c>
       <c r="D9" t="s">
         <v>57</v>
       </c>
-      <c r="E9" t="s">
-        <v>57</v>
+      <c r="E9" t="n">
+        <v>133.22</v>
       </c>
       <c r="F9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
-        <v>57</v>
+      <c r="G9" t="n">
+        <v>81.37</v>
       </c>
       <c r="H9" t="s">
         <v>57</v>
       </c>
-      <c r="I9" t="s">
-        <v>57</v>
+      <c r="I9" t="n">
+        <v>50.29</v>
       </c>
       <c r="J9" t="s">
         <v>57</v>
       </c>
-      <c r="K9" t="s">
-        <v>57</v>
+      <c r="K9" t="n">
+        <v>79.9</v>
       </c>
       <c r="L9" t="s">
         <v>57</v>
@@ -42776,32 +42776,32 @@
       <c r="B10" t="s">
         <v>57</v>
       </c>
-      <c r="C10" t="s">
-        <v>57</v>
+      <c r="C10" t="n">
+        <v>28.44</v>
       </c>
       <c r="D10" t="s">
         <v>57</v>
       </c>
-      <c r="E10" t="s">
-        <v>57</v>
+      <c r="E10" t="n">
+        <v>77.88</v>
       </c>
       <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="G10" t="s">
-        <v>57</v>
+      <c r="G10" t="n">
+        <v>74.94</v>
       </c>
       <c r="H10" t="s">
         <v>57</v>
       </c>
-      <c r="I10" t="s">
-        <v>57</v>
+      <c r="I10" t="n">
+        <v>22.2</v>
       </c>
       <c r="J10" t="s">
         <v>57</v>
       </c>
-      <c r="K10" t="s">
-        <v>57</v>
+      <c r="K10" t="n">
+        <v>54.45</v>
       </c>
       <c r="L10" t="s">
         <v>57</v>
@@ -42820,32 +42820,32 @@
       <c r="B11" t="s">
         <v>57</v>
       </c>
-      <c r="C11" t="s">
-        <v>57</v>
+      <c r="C11" t="n">
+        <v>28.98</v>
       </c>
       <c r="D11" t="s">
         <v>57</v>
       </c>
-      <c r="E11" t="s">
-        <v>57</v>
+      <c r="E11" t="n">
+        <v>84.16</v>
       </c>
       <c r="F11" t="s">
         <v>57</v>
       </c>
-      <c r="G11" t="s">
-        <v>57</v>
+      <c r="G11" t="n">
+        <v>41.36</v>
       </c>
       <c r="H11" t="s">
         <v>57</v>
       </c>
-      <c r="I11" t="s">
-        <v>57</v>
+      <c r="I11" t="n">
+        <v>33.16</v>
       </c>
       <c r="J11" t="s">
         <v>57</v>
       </c>
-      <c r="K11" t="s">
-        <v>57</v>
+      <c r="K11" t="n">
+        <v>47.21</v>
       </c>
       <c r="L11" t="s">
         <v>57</v>
@@ -42864,32 +42864,32 @@
       <c r="B12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
-        <v>57</v>
+      <c r="C12" t="n">
+        <v>20.07</v>
       </c>
       <c r="D12" t="s">
         <v>57</v>
       </c>
-      <c r="E12" t="s">
-        <v>57</v>
+      <c r="E12" t="n">
+        <v>60.06</v>
       </c>
       <c r="F12" t="s">
         <v>57</v>
       </c>
-      <c r="G12" t="s">
-        <v>57</v>
+      <c r="G12" t="n">
+        <v>32.32</v>
       </c>
       <c r="H12" t="s">
         <v>57</v>
       </c>
-      <c r="I12" t="s">
-        <v>57</v>
+      <c r="I12" t="n">
+        <v>25.24</v>
       </c>
       <c r="J12" t="s">
         <v>57</v>
       </c>
-      <c r="K12" t="s">
-        <v>57</v>
+      <c r="K12" t="n">
+        <v>34.73</v>
       </c>
       <c r="L12" t="s">
         <v>57</v>
@@ -42908,32 +42908,32 @@
       <c r="B13" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
-        <v>57</v>
+      <c r="C13" t="n">
+        <v>22.49</v>
       </c>
       <c r="D13" t="s">
         <v>57</v>
       </c>
-      <c r="E13" t="s">
-        <v>57</v>
+      <c r="E13" t="n">
+        <v>72.68</v>
       </c>
       <c r="F13" t="s">
         <v>57</v>
       </c>
-      <c r="G13" t="s">
-        <v>57</v>
+      <c r="G13" t="n">
+        <v>32.85</v>
       </c>
       <c r="H13" t="s">
         <v>57</v>
       </c>
-      <c r="I13" t="s">
-        <v>57</v>
+      <c r="I13" t="n">
+        <v>20.8</v>
       </c>
       <c r="J13" t="s">
         <v>57</v>
       </c>
-      <c r="K13" t="s">
-        <v>57</v>
+      <c r="K13" t="n">
+        <v>37.56</v>
       </c>
       <c r="L13" t="s">
         <v>57</v>
@@ -42952,32 +42952,32 @@
       <c r="B14" t="s">
         <v>57</v>
       </c>
-      <c r="C14" t="s">
-        <v>57</v>
+      <c r="C14" t="n">
+        <v>9.31</v>
       </c>
       <c r="D14" t="s">
         <v>57</v>
       </c>
-      <c r="E14" t="s">
-        <v>57</v>
+      <c r="E14" t="n">
+        <v>26.92</v>
       </c>
       <c r="F14" t="s">
         <v>57</v>
       </c>
-      <c r="G14" t="s">
-        <v>57</v>
+      <c r="G14" t="n">
+        <v>22.11</v>
       </c>
       <c r="H14" t="s">
         <v>57</v>
       </c>
-      <c r="I14" t="s">
-        <v>57</v>
+      <c r="I14" t="n">
+        <v>9.27</v>
       </c>
       <c r="J14" t="s">
         <v>57</v>
       </c>
-      <c r="K14" t="s">
-        <v>57</v>
+      <c r="K14" t="n">
+        <v>17.86</v>
       </c>
       <c r="L14" t="s">
         <v>57</v>
@@ -42996,32 +42996,32 @@
       <c r="B15" t="s">
         <v>57</v>
       </c>
-      <c r="C15" t="s">
-        <v>57</v>
+      <c r="C15" t="n">
+        <v>4.5</v>
       </c>
       <c r="D15" t="s">
         <v>57</v>
       </c>
-      <c r="E15" t="s">
-        <v>57</v>
+      <c r="E15" t="n">
+        <v>40.22</v>
       </c>
       <c r="F15" t="s">
         <v>57</v>
       </c>
-      <c r="G15" t="s">
-        <v>57</v>
+      <c r="G15" t="n">
+        <v>16.83</v>
       </c>
       <c r="H15" t="s">
         <v>57</v>
       </c>
-      <c r="I15" t="s">
-        <v>57</v>
+      <c r="I15" t="n">
+        <v>5.09</v>
       </c>
       <c r="J15" t="s">
         <v>57</v>
       </c>
-      <c r="K15" t="s">
-        <v>57</v>
+      <c r="K15" t="n">
+        <v>17.26</v>
       </c>
       <c r="L15" t="s">
         <v>57</v>
@@ -43040,32 +43040,32 @@
       <c r="B16" t="s">
         <v>57</v>
       </c>
-      <c r="C16" t="s">
-        <v>57</v>
+      <c r="C16" t="n">
+        <v>2.76</v>
       </c>
       <c r="D16" t="s">
         <v>57</v>
       </c>
-      <c r="E16" t="s">
-        <v>57</v>
+      <c r="E16" t="n">
+        <v>38.26</v>
       </c>
       <c r="F16" t="s">
         <v>57</v>
       </c>
-      <c r="G16" t="s">
-        <v>57</v>
+      <c r="G16" t="n">
+        <v>9.25</v>
       </c>
       <c r="H16" t="s">
         <v>57</v>
       </c>
-      <c r="I16" t="s">
-        <v>57</v>
+      <c r="I16" t="n">
+        <v>2.92</v>
       </c>
       <c r="J16" t="s">
         <v>57</v>
       </c>
-      <c r="K16" t="s">
-        <v>57</v>
+      <c r="K16" t="n">
+        <v>13.36</v>
       </c>
       <c r="L16" t="s">
         <v>57</v>

</xml_diff>